<commit_message>
Changing windoff ncao_iled from 1,5 to 5
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/BY_Trans.xlsx
+++ b/VerveStacks_EST/BY_Trans.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\VerveStacks\assumptions\VerveStacks_ISO_template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69D1EB1B-B45C-4149-AEE2-7B3180C9E8C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C9D1CEC-05CC-4910-8E8E-FEC68B75398E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="misc." sheetId="2" r:id="rId1"/>
@@ -618,23 +618,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{982CB9B3-DA63-443B-9AA5-BEE16CBC2D59}">
   <dimension ref="B3:L25"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="9.53125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.53125" customWidth="1"/>
-    <col min="4" max="4" width="9.73046875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="4.86328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.5703125" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="4.85546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:12" ht="17.649999999999999" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="3" spans="2:12" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="2:12" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="4" spans="2:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
         <v>0</v>
       </c>
@@ -669,7 +669,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>7</v>
       </c>
@@ -686,7 +686,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>4</v>
       </c>
@@ -697,7 +697,7 @@
         <v>8.76</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>8</v>
       </c>
@@ -714,7 +714,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>9</v>
       </c>
@@ -734,7 +734,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>38</v>
       </c>
@@ -751,7 +751,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>38</v>
       </c>
@@ -768,7 +768,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B11" s="3" t="s">
         <v>54</v>
       </c>
@@ -785,7 +785,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>39</v>
       </c>
@@ -805,7 +805,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>39</v>
       </c>
@@ -825,7 +825,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.45">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>47</v>
       </c>
@@ -839,12 +839,12 @@
         <v>2025</v>
       </c>
     </row>
-    <row r="20" spans="2:5" ht="17.649999999999999" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="20" spans="2:5" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B20" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="2:5" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="21" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="1" t="s">
         <v>0</v>
       </c>
@@ -858,7 +858,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>48</v>
       </c>
@@ -872,7 +872,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
         <v>48</v>
       </c>
@@ -886,7 +886,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>48</v>
       </c>
@@ -900,12 +900,12 @@
         <v>52</v>
       </c>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
         <v>48</v>
       </c>
       <c r="C25">
-        <v>1.5</v>
+        <v>5</v>
       </c>
       <c r="D25" t="s">
         <v>51</v>
@@ -922,23 +922,23 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84AA14F3-DC2C-40CD-9F35-1128DBBCBE73}">
   <dimension ref="B3:I15"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="13.265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.9296875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.46484375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.59765625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="59.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="59.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:9" ht="17.649999999999999" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="3" spans="2:9" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="2:9" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="4" spans="2:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
         <v>0</v>
       </c>
@@ -958,7 +958,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>23</v>
       </c>
@@ -975,7 +975,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>25</v>
       </c>
@@ -992,7 +992,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>25</v>
       </c>
@@ -1009,7 +1009,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>25</v>
       </c>
@@ -1026,7 +1026,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="9" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>30</v>
       </c>
@@ -1040,7 +1040,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>31</v>
       </c>
@@ -1057,12 +1057,12 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="2:9" ht="17.649999999999999" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="13" spans="2:9" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="14" spans="2:9" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="14" spans="2:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
         <v>6</v>
       </c>
@@ -1073,7 +1073,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>56</v>
       </c>

</xml_diff>

<commit_message>
Remove rcap_bnd from BY_Trans.xlsx
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/BY_Trans.xlsx
+++ b/VerveStacks_EST/BY_Trans.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\krraik\OneDrive - Tallinna Tehnikaülikool\Desktop\TIMES\safe_save\ee-times\VerveStacks_EST\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDBFABFD-40C6-40FE-B7A3-8D4DDA1F8273}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EEFCFF6-0CB3-4D1D-BBB7-5EB162299845}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -719,22 +719,19 @@
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>9</v>
-      </c>
-      <c r="D8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" t="s">
-        <v>11</v>
-      </c>
-      <c r="G8">
-        <v>4</v>
-      </c>
-      <c r="I8">
-        <v>0</v>
-      </c>
-      <c r="J8" t="s">
-        <v>14</v>
+        <v>37</v>
+      </c>
+      <c r="C8" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="H8">
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
@@ -744,48 +741,51 @@
       <c r="C9" t="s">
         <v>35</v>
       </c>
-      <c r="D9" s="3" t="s">
-        <v>44</v>
+      <c r="D9" t="s">
+        <v>45</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>36</v>
       </c>
       <c r="H9">
-        <v>40</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B10" t="s">
-        <v>37</v>
+      <c r="B10" s="3" t="s">
+        <v>53</v>
       </c>
       <c r="C10" t="s">
         <v>35</v>
       </c>
-      <c r="D10" t="s">
-        <v>45</v>
+      <c r="D10" s="3" t="s">
+        <v>44</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="H10">
-        <v>100</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B11" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="C11" t="s">
-        <v>35</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>52</v>
+      <c r="B11" t="s">
+        <v>38</v>
+      </c>
+      <c r="D11" t="s">
+        <v>39</v>
+      </c>
+      <c r="E11" t="s">
+        <v>42</v>
       </c>
       <c r="H11">
-        <v>0.9</v>
+        <v>0.95</v>
+      </c>
+      <c r="K11" t="s">
+        <v>41</v>
+      </c>
+      <c r="L11" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
@@ -793,13 +793,13 @@
         <v>38</v>
       </c>
       <c r="D12" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="E12" t="s">
         <v>42</v>
       </c>
       <c r="H12">
-        <v>0.95</v>
+        <v>0.85</v>
       </c>
       <c r="K12" t="s">
         <v>41</v>
@@ -810,44 +810,44 @@
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>38</v>
-      </c>
-      <c r="D13" t="s">
-        <v>43</v>
-      </c>
-      <c r="E13" t="s">
-        <v>42</v>
+        <v>46</v>
+      </c>
+      <c r="C13" t="s">
+        <v>35</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>51</v>
       </c>
       <c r="H13">
-        <v>0.85</v>
-      </c>
-      <c r="K13" t="s">
-        <v>41</v>
-      </c>
-      <c r="L13" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B14" t="s">
-        <v>46</v>
-      </c>
-      <c r="C14" t="s">
-        <v>35</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="H14">
         <v>2025</v>
       </c>
     </row>
-    <row r="20" spans="2:5" ht="18" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>9</v>
+      </c>
+      <c r="D17" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" t="s">
+        <v>11</v>
+      </c>
+      <c r="G17">
+        <v>4</v>
+      </c>
+      <c r="I17">
+        <v>0</v>
+      </c>
+      <c r="J17" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" spans="2:10" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B20" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="1" t="s">
         <v>0</v>
       </c>
@@ -861,7 +861,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>47</v>
       </c>
@@ -875,7 +875,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
         <v>47</v>
       </c>
@@ -889,7 +889,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>47</v>
       </c>
@@ -903,7 +903,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
         <v>47</v>
       </c>

</xml_diff>

<commit_message>
Changing start year of ele
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/BY_Trans.xlsx
+++ b/VerveStacks_EST/BY_Trans.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EEFCFF6-0CB3-4D1D-BBB7-5EB162299845}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7570B252-EE81-4208-A228-0994AF8D18CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -819,7 +819,7 @@
         <v>51</v>
       </c>
       <c r="H13">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="17" spans="2:10" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Changing start year of new investmeents
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/BY_Trans.xlsx
+++ b/VerveStacks_EST/BY_Trans.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7570B252-EE81-4208-A228-0994AF8D18CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A96D057E-5B52-4CFB-8BE2-905DDA9E49AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -819,7 +819,7 @@
         <v>51</v>
       </c>
       <c r="H13">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="17" spans="2:10" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Activating early retirements for oil shale
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/BY_Trans.xlsx
+++ b/VerveStacks_EST/BY_Trans.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A96D057E-5B52-4CFB-8BE2-905DDA9E49AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{874B7E55-AB2C-41FF-9155-3E31CC5F3EAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -822,32 +822,32 @@
         <v>2025</v>
       </c>
     </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B17" t="s">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
         <v>9</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D14" t="s">
         <v>12</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E14" t="s">
         <v>11</v>
       </c>
-      <c r="G17">
+      <c r="G14">
         <v>4</v>
       </c>
-      <c r="I17">
+      <c r="I14">
         <v>0</v>
       </c>
-      <c r="J17" t="s">
+      <c r="J14" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="2:10" ht="18" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:5" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B20" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="2:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="1" t="s">
         <v>0</v>
       </c>
@@ -861,7 +861,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>47</v>
       </c>
@@ -875,7 +875,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="23" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
         <v>47</v>
       </c>
@@ -889,7 +889,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="24" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>47</v>
       </c>
@@ -903,7 +903,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="25" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
         <v>47</v>
       </c>

</xml_diff>

<commit_message>
cap2act missing fix attempt
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/BY_Trans.xlsx
+++ b/VerveStacks_EST/BY_Trans.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87033A9E-F718-43F1-8BF0-C06252CD487F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00A1D548-0D6B-4399-9483-72D18801E633}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="misc." sheetId="2" r:id="rId1"/>
@@ -256,10 +256,10 @@
     <t>* Parameter values for qualifying technologies in each region, not tied to BASE</t>
   </si>
   <si>
-    <t>~TFM_UPD</t>
-  </si>
-  <si>
     <t>atrribute</t>
+  </si>
+  <si>
+    <t>TFM_UPD</t>
   </si>
 </sst>
 </file>
@@ -293,6 +293,8 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
+      <charset val="186"/>
     </font>
     <font>
       <b/>
@@ -390,7 +392,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="2"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1"/>
@@ -404,23 +406,12 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="3" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="3"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="3" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="3" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="3" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="3" quotePrefix="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="3" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
@@ -774,45 +765,45 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B3" s="21" t="s">
+      <c r="B3" s="7" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="22" t="s">
-        <v>74</v>
-      </c>
-      <c r="C4" s="22" t="s">
+      <c r="B4" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="C4" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="22" t="s">
+      <c r="D4" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="22" t="s">
+      <c r="E4" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="22" t="s">
+      <c r="F4" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="G4" s="22">
+      <c r="G4" s="15">
         <v>0</v>
       </c>
-      <c r="H4" s="22">
+      <c r="H4" s="15">
         <v>2022</v>
       </c>
-      <c r="I4" s="22">
+      <c r="I4" s="15">
         <v>2030</v>
       </c>
-      <c r="J4" s="22">
+      <c r="J4" s="15">
         <v>2035</v>
       </c>
-      <c r="K4" s="22" t="s">
+      <c r="K4" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="L4" s="22" t="s">
+      <c r="L4" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="M4" s="22" t="s">
+      <c r="M4" s="15" t="s">
         <v>20</v>
       </c>
     </row>
@@ -993,7 +984,6 @@
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
-      <c r="F20" s="11"/>
     </row>
     <row r="21" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="8" t="s">
@@ -1008,7 +998,6 @@
       <c r="E21" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="F21" s="11"/>
     </row>
     <row r="22" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
@@ -1023,7 +1012,6 @@
       <c r="E22" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="F22" s="11"/>
     </row>
     <row r="23" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
@@ -1272,160 +1260,160 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="3" spans="2:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="12"/>
-      <c r="I3" s="12"/>
-      <c r="J3" s="12"/>
-      <c r="K3" s="12"/>
-      <c r="L3" s="12"/>
-      <c r="M3" s="12"/>
-      <c r="N3" s="12"/>
-      <c r="O3" s="12"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
     </row>
     <row r="5" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B5" s="15" t="s">
-        <v>73</v>
-      </c>
-      <c r="C5" s="12"/>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12"/>
-      <c r="H5" s="14"/>
-      <c r="I5" s="13"/>
-      <c r="J5" s="13"/>
-      <c r="K5" s="13"/>
-      <c r="L5" s="13"/>
-      <c r="M5" s="13"/>
-      <c r="N5" s="13"/>
-      <c r="O5" s="13"/>
+      <c r="B5" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="5"/>
+      <c r="J5" s="5"/>
+      <c r="K5" s="5"/>
+      <c r="L5" s="5"/>
+      <c r="M5" s="5"/>
+      <c r="N5" s="5"/>
+      <c r="O5" s="5"/>
     </row>
     <row r="6" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="C6" s="16" t="s">
+      <c r="C6" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="D6" s="16" t="s">
+      <c r="D6" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="E6" s="16" t="s">
+      <c r="E6" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="F6" s="19" t="s">
+      <c r="F6" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="G6" s="19" t="s">
+      <c r="G6" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="H6" s="17" t="s">
+      <c r="H6" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="I6" s="17" t="s">
+      <c r="I6" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="J6" s="17" t="s">
+      <c r="J6" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="K6" s="17" t="s">
+      <c r="K6" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="L6" s="17" t="s">
+      <c r="L6" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="M6" s="17" t="s">
+      <c r="M6" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="N6" s="17" t="s">
+      <c r="N6" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="O6" s="17" t="s">
+      <c r="O6" s="11" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="7" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B7" s="20"/>
-      <c r="C7" s="20"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="20"/>
-      <c r="H7" s="12"/>
-      <c r="I7" s="12"/>
-      <c r="J7" s="20"/>
-      <c r="K7" s="20"/>
-      <c r="L7" s="20"/>
-      <c r="M7" s="20"/>
-      <c r="N7" s="20"/>
-      <c r="O7" s="20"/>
+      <c r="B7" s="14"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="4"/>
+      <c r="J7" s="14"/>
+      <c r="K7" s="14"/>
+      <c r="L7" s="14"/>
+      <c r="M7" s="14"/>
+      <c r="N7" s="14"/>
+      <c r="O7" s="14"/>
     </row>
     <row r="13" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B13" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="C13" s="12"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="12"/>
-      <c r="H13" s="14"/>
-      <c r="I13" s="13"/>
-      <c r="J13" s="13"/>
-      <c r="K13" s="13"/>
-      <c r="L13" s="13"/>
-      <c r="M13" s="13"/>
-      <c r="N13" s="13"/>
-      <c r="O13" s="13"/>
+      <c r="B13" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
+      <c r="H13" s="6"/>
+      <c r="I13" s="5"/>
+      <c r="J13" s="5"/>
+      <c r="K13" s="5"/>
+      <c r="L13" s="5"/>
+      <c r="M13" s="5"/>
+      <c r="N13" s="5"/>
+      <c r="O13" s="5"/>
     </row>
     <row r="14" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="16" t="s">
+      <c r="B14" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="C14" s="16" t="s">
+      <c r="C14" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="D14" s="16" t="s">
+      <c r="D14" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="E14" s="16" t="s">
+      <c r="E14" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="F14" s="19" t="s">
+      <c r="F14" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="G14" s="19" t="s">
+      <c r="G14" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="H14" s="17" t="s">
+      <c r="H14" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="I14" s="17" t="s">
+      <c r="I14" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="J14" s="17" t="s">
+      <c r="J14" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="K14" s="17" t="s">
+      <c r="K14" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="L14" s="17" t="s">
+      <c r="L14" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="M14" s="17" t="s">
+      <c r="M14" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="N14" s="17" t="s">
+      <c r="N14" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="O14" s="17" t="s">
+      <c r="O14" s="11" t="s">
         <v>71</v>
       </c>
     </row>

</xml_diff>

<commit_message>
by trans typo fix
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/BY_Trans.xlsx
+++ b/VerveStacks_EST/BY_Trans.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00A1D548-0D6B-4399-9483-72D18801E633}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C37353A1-726E-46DA-BC99-4EEFD7CF10A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="misc." sheetId="2" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="74">
   <si>
     <t>attribute</t>
   </si>
@@ -254,9 +254,6 @@
   </si>
   <si>
     <t>* Parameter values for qualifying technologies in each region, not tied to BASE</t>
-  </si>
-  <si>
-    <t>atrribute</t>
   </si>
   <si>
     <t>TFM_UPD</t>
@@ -771,7 +768,7 @@
     </row>
     <row r="4" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="15" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="C4" s="15" t="s">
         <v>5</v>
@@ -1279,7 +1276,7 @@
     </row>
     <row r="5" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B5" s="7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>

</xml_diff>

<commit_message>
trying to get rid of IMPNRGZ by seting pset_srt of ELE's START from 2025 to 2020
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/BY_Trans.xlsx
+++ b/VerveStacks_EST/BY_Trans.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C37353A1-726E-46DA-BC99-4EEFD7CF10A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E95EB259-2EA6-43CF-9EEB-50287FDA46E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="misc." sheetId="2" r:id="rId1"/>
@@ -951,7 +951,7 @@
         <v>50</v>
       </c>
       <c r="H13">
-        <v>2025</v>
+        <v>2020</v>
       </c>
     </row>
     <row r="14" spans="2:13" x14ac:dyDescent="0.25">

</xml_diff>